<commit_message>
Add articles found in her CV to the site and seed spreadsheet
Cross-checked her CV (سيرة ذاتية، تموز 2026) against the seed data;
verified and added 6 previously-missing academic articles published in
مجلة الحداثة (Al-Hadatha Magazine), 2008-2017 — each confirmed by byline
match on the publisher's own archive before adding.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Wadiha_El_Amiouni_Articles_and_Media.xlsx
+++ b/Wadiha_El_Amiouni_Articles_and_Media.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1260,6 +1260,156 @@
       <c r="E32" s="5" t="inlineStr">
         <is>
           <t>https://beirut2030.me/?p=5041</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>التعليم والتكنولوجيا في المؤسسات التربوية: استخدام التقنيات الحديثة في المدارس الخاصة</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>مجلة الحداثة / Al-Hadatha Magazine</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>2016-10-01</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>https://alhadathamagazine.blogspot.com/2016/12/blog-post.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>الإشكاليات النسوية ودورها في تأسيس علم اجتماع المرأة والإشكاليات الميدانية</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>مجلة الحداثة / Al-Hadatha Magazine</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>2016-01-01</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>https://alhadathamagazine.blogspot.com/2016/01/blog-post_26.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>التكاذب الافتراضي على مواقع التواصل الاجتماعي</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>مجلة الحداثة / Al-Hadatha Magazine</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>2017-04-01</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>https://alhadathamagazine.blogspot.com/2017/03/blog-post_13.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>المرأة العربية وجرائم الشرف</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>مجلة الحداثة / Al-Hadatha Magazine</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>2014-04-01</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>https://alhadathamagazine.blogspot.com/2014/01/blog-post.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>العنف في الخطاب السياسي العربي</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>مجلة الحداثة / Al-Hadatha Magazine</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>2012-07-01</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>https://alhadathamagazine.blogspot.com/2012/01/blog-post.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>المرأة في عصر النهضة</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>مجلة الحداثة / Al-Hadatha Magazine</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>2008-10-01</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>https://alhadathamagazine.blogspot.com/2008/01/blog-post.html</t>
         </is>
       </c>
     </row>
@@ -1298,6 +1448,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add General Security Magazine article (probable CV match)
Issue #107 (Aug 2022), topic and date match her CV citation exactly;
byline not visually confirmed since it's a scanned PDF. Flagged as a
probable match in the About/seed notes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Wadiha_El_Amiouni_Articles_and_Media.xlsx
+++ b/Wadiha_El_Amiouni_Articles_and_Media.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1410,6 +1410,31 @@
       <c r="E38" s="5" t="inlineStr">
         <is>
           <t>https://alhadathamagazine.blogspot.com/2008/01/blog-post.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>دور الحكومات الإلكترونية في محاربة الفساد</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>مجلة الأمن العام / General Security Magazine</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>2022-08-01</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>https://www.general-security.gov.lb/uploads/articles/10713.pdf</t>
         </is>
       </c>
     </row>
@@ -1454,6 +1479,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId37"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Sky News Arabia articles quoting her as a social researcher
4 pieces where she gives exclusive comment ("حديث خاص لموقع سكاي نيوز
عربية") — confirmed by name/quote match on each page before adding,
dates from page metadata (2021-2024).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Wadiha_El_Amiouni_Articles_and_Media.xlsx
+++ b/Wadiha_El_Amiouni_Articles_and_Media.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1435,6 +1435,106 @@
       <c r="E39" s="5" t="inlineStr">
         <is>
           <t>https://www.general-security.gov.lb/uploads/articles/10713.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>«القمار الإلكتروني».. آفة جديدة تنتشر بين شباب لبنان (تصريح)</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Sky News Arabia</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>2021-12-16</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>https://www.skynewsarabia.com/varieties/1486936-%D8%A7%D9%84%D9%82%D9%85%D8%A7%D8%B1-%D8%A7%D9%84%D8%A7%D9%95%D9%84%D9%83%D8%AA%D8%B1%D9%88%D9%86%D9%8A-%D8%A7%D9%93%D9%81%D8%A9-%D8%AC%D8%AF%D9%8A%D8%AF%D8%A9-%D8%AA%D9%86%D8%AA%D8%B4%D8%B1-%D8%B4%D8%A8%D8%A7%D8%A8-%D9%84%D8%A8%D9%86%D8%A7%D9%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>بينها 3 دول عربية.. ارتفاع معدل التعاسة في العالم (تصريح)</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Sky News Arabia</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>2022-10-20</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>https://www.skynewsarabia.com/varieties/1564444-%D8%A8%D9%8A%D9%86%D9%87%D8%A7-3-%D8%AF%D9%88%D9%84-%D8%B9%D8%B1%D8%A8%D9%8A%D8%A9-%D8%A7%D8%B1%D8%AA%D9%81%D8%A7%D8%B9-%D9%85%D8%B9%D8%AF%D9%84-%D8%A7%D9%84%D8%AA%D8%B9%D8%A7%D8%B3%D8%A9-%D8%A7%D9%84%D8%B9%D8%A7%D9%84%D9%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>في رحيل سنة 2021.. الأزمات تطوق اللبنانيين من كل جانب (تصريح)</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Sky News Arabia</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>2021-12-28</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>https://www.skynewsarabia.com/middle-east/1489717-%D8%B1%D8%AD%D9%8A%D9%84-%D8%B3%D9%86%D8%A9-2021-%D8%A7%D9%84%D8%A7%D9%94%D8%B2%D9%85%D8%A7%D8%AA-%D8%AA%D8%B7%D9%88%D9%82-%D8%A7%D9%84%D9%84%D8%A8%D9%86%D8%A7%D9%86%D9%8A%D9%8A%D9%86-%D9%83%D9%84-%D8%AC%D8%A7%D9%86%D8%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>أطفال لبنان بين «تروما الغارات» والدراسة الحضورية (تصريح)</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Sky News Arabia</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>2024-11-13</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>https://www.skynewsarabia.com/middle-east/1754839-%D8%A7%D9%94%D8%B7%D9%81%D8%A7%D9%84-%D9%84%D8%A8%D9%86%D8%A7%D9%86-%D8%AA%D8%B1%D9%88%D9%85%D8%A7-%D8%A7%D9%84%D8%BA%D8%A7%D8%B1%D8%A7%D8%AA-%D9%88%D8%A7%D9%84%D8%AF%D8%B1%D8%A7%D8%B3%D8%A9-%D8%A7%D9%84%D8%AD%D8%B6%D9%88%D8%B1%D9%8A%D8%A9</t>
         </is>
       </c>
     </row>
@@ -1480,6 +1580,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId41"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Statement (تصريح) content type; reclassify press-quote pieces
New third content type alongside Articles and Media, for press pieces
that quote her commentary rather than being authored by her.

- Schema: add "statement" to the item_type enum (pushed to Neon)
- Pages: /statements browse page + a third home rail; nav + footer links
- Admin: 3-way type toggle (مقال | ظهور إعلامي | تصريح) + 💬 list icon
- Cards: "قراءة التصريح / Read statement" CTA; statements render like
  articles (no play glyph, no format filter)
- i18n: statement keys in both ar/en
- Reclassified 5 existing quote items (4 Sky News Arabia + Beirut 2030)
  from article → statement and stripped the "(تصريح)" title suffix
- Seed: new "Statements تصريح" sheet in the spreadsheet + seed.ts reader

Verified in browser (AR + EN, /statements + admin toggle) and via an
adversarial review pass (7 candidate findings, 0 confirmed).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Wadiha_El_Amiouni_Articles_and_Media.xlsx
+++ b/Wadiha_El_Amiouni_Articles_and_Media.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet name="Articles مقالات" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Media ظهور إعلامي" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="About" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Statements تصريح" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="About" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -469,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1244,22 +1245,22 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>كيف يفهم الأطفال الموت... وكيف ندعمهم في مواجهة فقدان القريب؟ (تصريح)</t>
+          <t>التعليم والتكنولوجيا في المؤسسات التربوية: استخدام التقنيات الحديثة في المدارس الخاصة</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Beirut 2030</t>
+          <t>مجلة الحداثة / Al-Hadatha Magazine</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2016-10-01</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>https://beirut2030.me/?p=5041</t>
+          <t>https://alhadathamagazine.blogspot.com/2016/12/blog-post.html</t>
         </is>
       </c>
     </row>
@@ -1269,7 +1270,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>التعليم والتكنولوجيا في المؤسسات التربوية: استخدام التقنيات الحديثة في المدارس الخاصة</t>
+          <t>الإشكاليات النسوية ودورها في تأسيس علم اجتماع المرأة والإشكاليات الميدانية</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -1279,12 +1280,12 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>2016-10-01</t>
+          <t>2016-01-01</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>https://alhadathamagazine.blogspot.com/2016/12/blog-post.html</t>
+          <t>https://alhadathamagazine.blogspot.com/2016/01/blog-post_26.html</t>
         </is>
       </c>
     </row>
@@ -1294,7 +1295,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>الإشكاليات النسوية ودورها في تأسيس علم اجتماع المرأة والإشكاليات الميدانية</t>
+          <t>التكاذب الافتراضي على مواقع التواصل الاجتماعي</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -1304,12 +1305,12 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>2016-01-01</t>
+          <t>2017-04-01</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>https://alhadathamagazine.blogspot.com/2016/01/blog-post_26.html</t>
+          <t>https://alhadathamagazine.blogspot.com/2017/03/blog-post_13.html</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1320,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>التكاذب الافتراضي على مواقع التواصل الاجتماعي</t>
+          <t>المرأة العربية وجرائم الشرف</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -1329,12 +1330,12 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>2017-04-01</t>
+          <t>2014-04-01</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>https://alhadathamagazine.blogspot.com/2017/03/blog-post_13.html</t>
+          <t>https://alhadathamagazine.blogspot.com/2014/01/blog-post.html</t>
         </is>
       </c>
     </row>
@@ -1344,7 +1345,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>المرأة العربية وجرائم الشرف</t>
+          <t>العنف في الخطاب السياسي العربي</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -1354,12 +1355,12 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>2014-04-01</t>
+          <t>2012-07-01</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>https://alhadathamagazine.blogspot.com/2014/01/blog-post.html</t>
+          <t>https://alhadathamagazine.blogspot.com/2012/01/blog-post.html</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1370,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>العنف في الخطاب السياسي العربي</t>
+          <t>المرأة في عصر النهضة</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -1379,12 +1380,12 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>2012-07-01</t>
+          <t>2008-10-01</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>https://alhadathamagazine.blogspot.com/2012/01/blog-post.html</t>
+          <t>https://alhadathamagazine.blogspot.com/2008/01/blog-post.html</t>
         </is>
       </c>
     </row>
@@ -1394,147 +1395,22 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>المرأة في عصر النهضة</t>
+          <t>دور الحكومات الإلكترونية في محاربة الفساد</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>مجلة الحداثة / Al-Hadatha Magazine</t>
+          <t>مجلة الأمن العام / General Security Magazine</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>2008-10-01</t>
+          <t>2022-08-01</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>https://alhadathamagazine.blogspot.com/2008/01/blog-post.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="n">
-        <v>37</v>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>دور الحكومات الإلكترونية في محاربة الفساد</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>مجلة الأمن العام / General Security Magazine</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>2022-08-01</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
           <t>https://www.general-security.gov.lb/uploads/articles/10713.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="n">
-        <v>38</v>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>«القمار الإلكتروني».. آفة جديدة تنتشر بين شباب لبنان (تصريح)</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>Sky News Arabia</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>2021-12-16</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>https://www.skynewsarabia.com/varieties/1486936-%D8%A7%D9%84%D9%82%D9%85%D8%A7%D8%B1-%D8%A7%D9%84%D8%A7%D9%95%D9%84%D9%83%D8%AA%D8%B1%D9%88%D9%86%D9%8A-%D8%A7%D9%93%D9%81%D8%A9-%D8%AC%D8%AF%D9%8A%D8%AF%D8%A9-%D8%AA%D9%86%D8%AA%D8%B4%D8%B1-%D8%B4%D8%A8%D8%A7%D8%A8-%D9%84%D8%A8%D9%86%D8%A7%D9%86</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="3" t="n">
-        <v>39</v>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>بينها 3 دول عربية.. ارتفاع معدل التعاسة في العالم (تصريح)</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>Sky News Arabia</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>2022-10-20</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>https://www.skynewsarabia.com/varieties/1564444-%D8%A8%D9%8A%D9%86%D9%87%D8%A7-3-%D8%AF%D9%88%D9%84-%D8%B9%D8%B1%D8%A8%D9%8A%D8%A9-%D8%A7%D8%B1%D8%AA%D9%81%D8%A7%D8%B9-%D9%85%D8%B9%D8%AF%D9%84-%D8%A7%D9%84%D8%AA%D8%B9%D8%A7%D8%B3%D8%A9-%D8%A7%D9%84%D8%B9%D8%A7%D9%84%D9%85</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>في رحيل سنة 2021.. الأزمات تطوق اللبنانيين من كل جانب (تصريح)</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>Sky News Arabia</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>2021-12-28</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>https://www.skynewsarabia.com/middle-east/1489717-%D8%B1%D8%AD%D9%8A%D9%84-%D8%B3%D9%86%D8%A9-2021-%D8%A7%D9%84%D8%A7%D9%94%D8%B2%D9%85%D8%A7%D8%AA-%D8%AA%D8%B7%D9%88%D9%82-%D8%A7%D9%84%D9%84%D8%A8%D9%86%D8%A7%D9%86%D9%8A%D9%8A%D9%86-%D9%83%D9%84-%D8%AC%D8%A7%D9%86%D8%A8</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="3" t="n">
-        <v>41</v>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>أطفال لبنان بين «تروما الغارات» والدراسة الحضورية (تصريح)</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>Sky News Arabia</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>2024-11-13</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>https://www.skynewsarabia.com/middle-east/1754839-%D8%A7%D9%94%D8%B7%D9%81%D8%A7%D9%84-%D9%84%D8%A8%D9%86%D8%A7%D9%86-%D8%AA%D8%B1%D9%88%D9%85%D8%A7-%D8%A7%D9%84%D8%BA%D8%A7%D8%B1%D8%A7%D8%AA-%D9%88%D8%A7%D9%84%D8%AF%D8%B1%D8%A7%D8%B3%D8%A9-%D8%A7%D9%84%D8%AD%D8%B6%D9%88%D8%B1%D9%8A%D8%A9</t>
         </is>
       </c>
     </row>
@@ -1579,11 +1455,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId41"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2669,6 +2540,196 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>تصريحات صحفية لـ أ.د. وديعة الأميوني — Press statements</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>العنوان / Title</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>المصدر / Source</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>التاريخ / Date</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>الرابط / Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>كيف يفهم الأطفال الموت... وكيف ندعمهم في مواجهة فقدان القريب؟</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Beirut 2030</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>https://beirut2030.me/?p=5041</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>«القمار الإلكتروني».. آفة جديدة تنتشر بين شباب لبنان</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Sky News Arabia</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>2021-12-16</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>https://www.skynewsarabia.com/varieties/1486936-%D8%A7%D9%84%D9%82%D9%85%D8%A7%D8%B1-%D8%A7%D9%84%D8%A7%D9%95%D9%84%D9%83%D8%AA%D8%B1%D9%88%D9%86%D9%8A-%D8%A7%D9%93%D9%81%D8%A9-%D8%AC%D8%AF%D9%8A%D8%AF%D8%A9-%D8%AA%D9%86%D8%AA%D8%B4%D8%B1-%D8%B4%D8%A8%D8%A7%D8%A8-%D9%84%D8%A8%D9%86%D8%A7%D9%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>بينها 3 دول عربية.. ارتفاع معدل التعاسة في العالم</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Sky News Arabia</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>2022-10-20</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>https://www.skynewsarabia.com/varieties/1564444-%D8%A8%D9%8A%D9%86%D9%87%D8%A7-3-%D8%AF%D9%88%D9%84-%D8%B9%D8%B1%D8%A8%D9%8A%D8%A9-%D8%A7%D8%B1%D8%AA%D9%81%D8%A7%D8%B9-%D9%85%D8%B9%D8%AF%D9%84-%D8%A7%D9%84%D8%AA%D8%B9%D8%A7%D8%B3%D8%A9-%D8%A7%D9%84%D8%B9%D8%A7%D9%84%D9%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>في رحيل سنة 2021.. الأزمات تطوق اللبنانيين من كل جانب</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Sky News Arabia</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>2021-12-28</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>https://www.skynewsarabia.com/middle-east/1489717-%D8%B1%D8%AD%D9%8A%D9%84-%D8%B3%D9%86%D8%A9-2021-%D8%A7%D9%84%D8%A7%D9%94%D8%B2%D9%85%D8%A7%D8%AA-%D8%AA%D8%B7%D9%88%D9%82-%D8%A7%D9%84%D9%84%D8%A8%D9%86%D8%A7%D9%86%D9%8A%D9%8A%D9%86-%D9%83%D9%84-%D8%AC%D8%A7%D9%86%D8%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>أطفال لبنان بين «تروما الغارات» والدراسة الحضورية</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Sky News Arabia</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>2024-11-13</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>https://www.skynewsarabia.com/middle-east/1754839-%D8%A7%D9%94%D8%B7%D9%81%D8%A7%D9%84-%D9%84%D8%A8%D9%86%D8%A7%D9%86-%D8%AA%D8%B1%D9%88%D9%85%D8%A7-%D8%A7%D9%84%D8%BA%D8%A7%D8%B1%D8%A7%D8%AA-%D9%88%D8%A7%D9%84%D8%AF%D8%B1%D8%A7%D8%B3%D8%A9-%D8%A7%D9%84%D8%AD%D8%B6%D9%88%D8%B1%D9%8A%D8%A9</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId5"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Add 12 statements: Alhurra commentary + conference/university participation
Found via Firecrawl sweep of alhurra.com and Lebanese-University /
Balamand / Altaleb / NNA / Ecco Watan / Sawt el Jil coverage. Each
verified to quote her as speaker, organizer, or commentator (byline /
name confirmed on the publisher's own page). Deduped to one
authoritative source per event.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Wadiha_El_Amiouni_Articles_and_Media.xlsx
+++ b/Wadiha_El_Amiouni_Articles_and_Media.xlsx
@@ -2540,7 +2540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2709,6 +2709,306 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>أطفال لبنان.. كوابيس الحرب لا تعرف الهدنة</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>الحرة / Alhurra</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>https://alhurra.com/7919</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>أمطرت في طهران ففتح لبنان المظلّة</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>الحرة / Alhurra</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>https://alhurra.com/10950</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>مؤتمر «استراتيجيّات التحوّل الرقمي والحوكمة الرشيدة في لبنان» في جامعة البلمند</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>جامعة البلمند / University of Balamand</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>2023-02-23</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>http://www.balamand.edu.lb/news/AllNews/Pages/Details.aspx?FilterField1=ID&amp;FilterValue1=325</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>مؤتمر جمعية «جاد» في اليوم العالمي للحد من التدخين</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>الوكالة الوطنية للإعلام / NNA</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>2024-05-31</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>https://www.nna-leb.gov.lb/ar/news/294245</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>ندوة «الإعلام في زمن الحروب» في طرابلس بمشاركة مكاري</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>إيكو وطن / Ecco Watan</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>2024-03-12</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>https://www.eccowatan.com/pages/48664</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>ندوة «دور المرأة في التربية على المواطنية» في مركز الصفدي - طرابلس</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>صوت الجيل / Sawt el Jil</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>2025-02-18</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>https://sawteljil.com/id/12545</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>طلاب العلوم الاجتماعية (3) ينهون تدريبًا حول «إدارة السمعة الرقمية»</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>الجامعة اللبنانية / Lebanese University</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>2024-01-18</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>https://ul.edu.lb/ar/node/6357</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>ورشة تدريبية في معهد العلوم الإجتماعية (3) حول بناء وتطوير القدرات البشرية والمؤسسية</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>موقع الطالب / Altaleb</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>2024-01-15</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>https://altaleb.org.lb/%D9%88%D8%B1%D8%B4%D8%A9-%D8%AA%D8%AF%D8%B1%D9%8A%D8%A8%D9%8A%D8%A9-%D9%81%D9%8A-%D9%85%D8%B9%D9%87%D8%AF-%D8%A7%D9%84%D8%B9%D9%84%D9%88%D9%85-%D8%A7%D9%84%D8%A5%D8%AC%D8%AA%D9%85%D8%A7%D8%B9%D9%8A/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>إطلاق «نادي الكتاب» في معهد العلوم الإجتماعية (3)</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>موقع الطالب / Altaleb</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>2024-01-29</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>https://altaleb.org.lb/%D8%A5%D8%B7%D9%84%D8%A7%D9%82-%D9%86%D8%A7%D8%AF%D9%8A-%D8%A7%D9%84%D9%83%D8%AA%D8%A7%D8%A8-%D9%81%D9%8A-%D9%85%D8%B9%D9%87%D8%AF-%D8%A7%D9%84%D8%B9%D9%84%D9%88%D9%85-%D8%A7%D9%84%D8%A5/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>جلسة حقوقية حول «قانون العمل اللبناني» في معهد العلوم الاجتماعية (3)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>الجامعة اللبنانية / Lebanese University</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>https://ul.edu.lb/ar/node/6246</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>معهد العلوم الاجتماعية (3) يشارك في يوم توجيهي لطلاب المرحلة الثانوية</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>الجامعة اللبنانية / Lebanese University</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>https://ul.edu.lb/ar/node/6205</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>حملة تشجير في معهد العلوم الاجتماعية (3)</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>الجامعة اللبنانية / Lebanese University</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>https://ul.edu.lb/ar/%D8%AD%D9%85%D9%84%D8%A9-%D8%AA%D8%B4%D8%AC%D9%8A%D8%B1-%D9%81%D9%8A-%D9%85%D8%B9%D9%87%D8%AF-%D8%A7%D9%84%D8%B9%D9%84%D9%88%D9%85-%D8%A7%D9%84%D8%A7%D8%AC%D8%AA%D9%85%D8%A7%D8%B9%D9%8A%D8%A9-3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
@@ -2719,6 +3019,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 4 more participation items to Statements (delegate/appearance coverage)
Two conferences she attended representing MP Frangieh (JUS blended-
learning conf, second North AI-in-education conf), her institute-
director appointment, and a Red Cross awareness activity she opened.
Deduped against existing items; excluded her CV/profile pages and a
duplicate of the الإعلام في زمن الحروب seminar.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Wadiha_El_Amiouni_Articles_and_Media.xlsx
+++ b/Wadiha_El_Amiouni_Articles_and_Media.xlsx
@@ -2540,7 +2540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3006,6 +3006,106 @@
       <c r="E19" s="5" t="inlineStr">
         <is>
           <t>https://ul.edu.lb/ar/%D8%AD%D9%85%D9%84%D8%A9-%D8%AA%D8%B4%D8%AC%D9%8A%D8%B1-%D9%81%D9%8A-%D9%85%D8%B9%D9%87%D8%AF-%D8%A7%D9%84%D8%B9%D9%84%D9%88%D9%85-%D8%A7%D9%84%D8%A7%D8%AC%D8%AA%D9%85%D8%A7%D8%B9%D9%8A%D8%A9-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>ممثلةً النائب فرنجيه في المؤتمر الدولي المدمج «معايير جودة التعليم عن بُعد» في اليسوعية</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>المرده / Elmarada</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>2025-01-23</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>https://elmarada.org/%D8%A7%D9%84%D8%AF%D9%83%D8%AA%D9%88%D8%B1%D8%A9-%D9%88%D8%AF%D9%8A%D8%B9%D8%A9-%D8%A7%D9%84%D8%A3%D9%85%D9%8A%D9%88%D9%86%D9%8A-%D9%85%D9%85%D8%AB%D9%84%D8%A9%D9%8B-%D8%A7%D9%84%D9%86%D8%A7%D8%A6/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>ممثلةً النائب فرنجيه في المؤتمر الثاني في الشمال «تكنولوجيا الإدارة والتعليم والذكاء الاصطناعي»</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>المرده / Elmarada</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>2025-07-25</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>https://elmarada.org/%D9%88%D8%AF%D9%8A%D8%B9%D8%A9-%D8%A7%D9%84%D8%A3%D9%85%D9%8A%D9%88%D9%86%D9%8A-%D9%85%D9%85%D8%AB%D9%84%D8%A9-%D8%A7%D9%84%D9%86%D8%A7%D8%A6%D8%A8-%D9%81%D8%B1%D9%86%D8%AC%D9%8A%D9%87-%D9%81%D9%8A/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>البروفسورة وديعة الأميوني تتسلّم مهام مديرة معهد العلوم الاجتماعية – الفرع الثالث</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>ستار نيوز فيجن / Star News Vision</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>2023-05-14</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>https://starnewsvision.com/2023/05/14/%D8%A7%D9%84%D8%A8%D8%B1%D9%88%D9%81%D8%B3%D9%88%D8%B1%D8%A9-%D9%88%D8%AF%D9%8A%D8%B9%D8%A9-%D8%A7%D9%84%D8%A3%D9%85%D9%8A%D9%88%D9%86%D9%8A-%D8%AA%D8%AA%D8%B3%D9%84%D9%85-%D9%85%D9%87%D8%A7%D9%85/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>نشاط توعوي للصليب الأحمر اللبناني في معهد العلوم الاجتماعية (3)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>الوكالة الوطنية للإعلام / NNA</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>https://www.nna-leb.gov.lb/ar/news/414663</t>
         </is>
       </c>
     </row>
@@ -3031,6 +3131,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove two elmarada delegate-coverage items from Statements
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Wadiha_El_Amiouni_Articles_and_Media.xlsx
+++ b/Wadiha_El_Amiouni_Articles_and_Media.xlsx
@@ -2540,7 +2540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3015,22 +3015,22 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>ممثلةً النائب فرنجيه في المؤتمر الدولي المدمج «معايير جودة التعليم عن بُعد» في اليسوعية</t>
+          <t>البروفسورة وديعة الأميوني تتسلّم مهام مديرة معهد العلوم الاجتماعية – الفرع الثالث</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>المرده / Elmarada</t>
+          <t>ستار نيوز فيجن / Star News Vision</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>2025-01-23</t>
+          <t>2023-05-14</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>https://elmarada.org/%D8%A7%D9%84%D8%AF%D9%83%D8%AA%D9%88%D8%B1%D8%A9-%D9%88%D8%AF%D9%8A%D8%B9%D8%A9-%D8%A7%D9%84%D8%A3%D9%85%D9%8A%D9%88%D9%86%D9%8A-%D9%85%D9%85%D8%AB%D9%84%D8%A9%D9%8B-%D8%A7%D9%84%D9%86%D8%A7%D8%A6/</t>
+          <t>https://starnewsvision.com/2023/05/14/%D8%A7%D9%84%D8%A8%D8%B1%D9%88%D9%81%D8%B3%D9%88%D8%B1%D8%A9-%D9%88%D8%AF%D9%8A%D8%B9%D8%A9-%D8%A7%D9%84%D8%A3%D9%85%D9%8A%D9%88%D9%86%D9%8A-%D8%AA%D8%AA%D8%B3%D9%84%D9%85-%D9%85%D9%87%D8%A7%D9%85/</t>
         </is>
       </c>
     </row>
@@ -3040,70 +3040,20 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>ممثلةً النائب فرنجيه في المؤتمر الثاني في الشمال «تكنولوجيا الإدارة والتعليم والذكاء الاصطناعي»</t>
+          <t>نشاط توعوي للصليب الأحمر اللبناني في معهد العلوم الاجتماعية (3)</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>المرده / Elmarada</t>
+          <t>الوكالة الوطنية للإعلام / NNA</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>2025-07-25</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>https://elmarada.org/%D9%88%D8%AF%D9%8A%D8%B9%D8%A9-%D8%A7%D9%84%D8%A3%D9%85%D9%8A%D9%88%D9%86%D9%8A-%D9%85%D9%85%D8%AB%D9%84%D8%A9-%D8%A7%D9%84%D9%86%D8%A7%D8%A6%D8%A8-%D9%81%D8%B1%D9%86%D8%AC%D9%8A%D9%87-%D9%81%D9%8A/</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>البروفسورة وديعة الأميوني تتسلّم مهام مديرة معهد العلوم الاجتماعية – الفرع الثالث</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>ستار نيوز فيجن / Star News Vision</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>2023-05-14</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>https://starnewsvision.com/2023/05/14/%D8%A7%D9%84%D8%A8%D8%B1%D9%88%D9%81%D8%B3%D9%88%D8%B1%D8%A9-%D9%88%D8%AF%D9%8A%D8%B9%D8%A9-%D8%A7%D9%84%D8%A3%D9%85%D9%8A%D9%88%D9%86%D9%8A-%D8%AA%D8%AA%D8%B3%D9%84%D9%85-%D9%85%D9%87%D8%A7%D9%85/</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>نشاط توعوي للصليب الأحمر اللبناني في معهد العلوم الاجتماعية (3)</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>الوكالة الوطنية للإعلام / NNA</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>2026-02-20</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>https://www.nna-leb.gov.lb/ar/news/414663</t>
         </is>
@@ -3133,8 +3083,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>